<commit_message>
Use empty PRISM wheel as PRISM Brain Mapping hero (#5)
Replace the hero photo on prism-brain-mapping.html with the empty
four-colour PRISM wheel from the owner's 6_Puste_Koło_PRISM.pdf:
a 400 dpi render cropped to the wheel and its eight labels on white,
with 640/1000/1400 px square WebP variants, a new alt text and matching
width/height. check_site.py knows the PRISM hero size, the Excel
template is regenerated (only the e046 alt row changed) and the render
is documented in docs/source-mapping.md and HANDOFF.md.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/teksty-strony.xlsx
+++ b/teksty-strony.xlsx
@@ -12499,14 +12499,14 @@
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>Katarzyna Chałas - coach</t>
+          <t>Puste koło PRISM Brain Mapping w czterech kolorach</t>
         </is>
       </c>
       <c r="F305" s="4" t="inlineStr"/>
       <c r="G305" s="5" t="inlineStr"/>
       <c r="H305" s="2" t="inlineStr">
         <is>
-          <t>img[data-content-id="e046"] | assets/hero-1000.webp</t>
+          <t>img[data-content-id="e046"] | assets/hero-prism-1000.webp</t>
         </is>
       </c>
       <c r="I305" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Use MTQ Plus logo as MTQ Plus hero (#4)
Replace the hero photo on mtq-plus.html with the MTQ Plus logo from the
owner's 4.png (500 × 500 px). The transparent background is flattened
onto white without scaling, cropping or retouching and saved as a
lossless WebP (5 KB, pixel-identical), so the decorative frame stays
hidden behind the image. img and preload get the new src/srcset (single
500w candidate), 500 × 500 width/height and the alt "Logo badania MTQ
Plus". check_site.py knows the MTQ Plus hero size, the Excel template is
regenerated (only the e046 alt row changed) and the source, conversion
and 2× softness (next_steps card 1925) are documented in
docs/source-mapping.md and HANDOFF.md.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/teksty-strony.xlsx
+++ b/teksty-strony.xlsx
@@ -13747,14 +13747,14 @@
       </c>
       <c r="E337" s="2" t="inlineStr">
         <is>
-          <t>Katarzyna Chałas - coach</t>
+          <t>Logo badania MTQ Plus</t>
         </is>
       </c>
       <c r="F337" s="4" t="inlineStr"/>
       <c r="G337" s="5" t="inlineStr"/>
       <c r="H337" s="2" t="inlineStr">
         <is>
-          <t>img[data-content-id="e046"] | assets/hero-1000.webp</t>
+          <t>img[data-content-id="e046"] | assets/hero-mtq-plus.webp</t>
         </is>
       </c>
       <c r="I337" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Remove sample PRISM map from PRISM Brain Mapping page
Owner asked to remove the graphic (card 1931, phone screenshot): drop
figure.prism-map with its full-size link and source caption, both map
files, the .prism-map styles and the map rows of teksty-strony.xlsx
(373 -> 368). check_site.py now guards against the map returning.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/teksty-strony.xlsx
+++ b/teksty-strony.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teksty" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Teksty'!$A$1:$I$374</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Teksty'!$A$1:$I$369</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -598,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I374"/>
+  <dimension ref="A1:I369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11894,7 +11894,7 @@
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e056:href</t>
+          <t>prism-brain-mapping:e060:text</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
@@ -11909,31 +11909,31 @@
       </c>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t>https://prismbrainmapping.pl/wp-content/uploads/2020/07/mapa-prism-brain-mapping.png</t>
+          <t>Co pokazuje PRISM Brain Mapping?</t>
         </is>
       </c>
       <c r="F290" s="4" t="inlineStr"/>
       <c r="G290" s="5" t="inlineStr"/>
       <c r="H290" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e056"] |  → https://prismbrainmapping.pl/wp-content/uploads/2020/07/mapa-prism-brain-mapping.png</t>
+          <t>h2[data-content-id="e060"]</t>
         </is>
       </c>
       <c r="I290" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e056:aria-label</t>
+          <t>prism-brain-mapping:e061:text</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
@@ -11948,31 +11948,31 @@
       </c>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>Etykieta dostępności</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E291" s="2" t="inlineStr">
         <is>
-          <t>Otwórz mapę PRISM w pełnym rozmiarze</t>
+          <t>Badanie odbywa się online i polega na udzieleniu odpowiedzi na kilkadziesiąt pytań. Na ich podstawie powstaje indywidualny profil przedstawiający 8 typów preferowanych zachowań oraz ich natężenie. PRISM pozwala również przyjrzeć się 26 czynnikom związanym z zachowaniem badanej osoby w określonych sytuacjach.</t>
         </is>
       </c>
       <c r="F291" s="4" t="inlineStr"/>
       <c r="G291" s="5" t="inlineStr"/>
       <c r="H291" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e056"] |  → https://prismbrainmapping.pl/wp-content/uploads/2020/07/mapa-prism-brain-mapping.png</t>
+          <t>p[data-content-id="e061"]</t>
         </is>
       </c>
       <c r="I291" s="2" t="inlineStr">
         <is>
-          <t>aria-label</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e057:alt</t>
+          <t>prism-brain-mapping:e063:text</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
@@ -11987,31 +11987,31 @@
       </c>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>Opis obrazu (alt)</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr">
         <is>
-          <t>Mapa PRISM Brain Mapping przedstawiająca osiem preferencji zachowań w czterech kolorach</t>
+          <t>Najbardziej charakterystycznym elementem badania jest mapa PRISM – przejrzysta wizualizacja, która pomaga zobaczyć własny profil psychologiczny z różnych perspektyw. Pokazuje między innymi naturalne preferencje zachowania, sposób, w jaki dostosowujemy się do wymagań otoczenia, oraz wzorzec zachowania, który najczęściej prezentujemy w relacjach z innymi.</t>
         </is>
       </c>
       <c r="F292" s="4" t="inlineStr"/>
       <c r="G292" s="5" t="inlineStr"/>
       <c r="H292" s="2" t="inlineStr">
         <is>
-          <t>img[data-content-id="e057"] | assets/mapa-prism-brain-mapping.webp</t>
+          <t>p[data-content-id="e063"]</t>
         </is>
       </c>
       <c r="I292" s="2" t="inlineStr">
         <is>
-          <t>alt</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e058:text</t>
+          <t>prism-brain-mapping:e065:text</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
@@ -12026,19 +12026,19 @@
       </c>
       <c r="D293" s="2" t="inlineStr">
         <is>
-          <t>Podpis ilustracji</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E293" s="2" t="inlineStr">
         <is>
-          <t>Źródło: prismbrainmapping.pl</t>
+          <t>PRISM dostarcza także informacji dotyczących inteligencji emocjonalnej, odporności psychicznej oraz cech osobowości w modelu Wielkiej Piątki. Dzięki temu pozwala szerzej spojrzeć na własne funkcjonowanie i dostrzec zarówno mocne strony, jak i obszary, które mogą wymagać większej uwagi.</t>
         </is>
       </c>
       <c r="F293" s="4" t="inlineStr"/>
       <c r="G293" s="5" t="inlineStr"/>
       <c r="H293" s="2" t="inlineStr">
         <is>
-          <t>figcaption[data-content-id="e058"]</t>
+          <t>p[data-content-id="e065"]</t>
         </is>
       </c>
       <c r="I293" s="2" t="inlineStr">
@@ -12050,7 +12050,7 @@
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e059:href</t>
+          <t>prism-brain-mapping:e068:text</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
@@ -12065,31 +12065,31 @@
       </c>
       <c r="D294" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
-          <t>https://prismbrainmapping.pl/</t>
+          <t>Po co wykonywać PRISM Brain Mapping?</t>
         </is>
       </c>
       <c r="F294" s="4" t="inlineStr"/>
       <c r="G294" s="5" t="inlineStr"/>
       <c r="H294" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e059"] | prismbrainmapping.pl → https://prismbrainmapping.pl/</t>
+          <t>h2[data-content-id="e068"]</t>
         </is>
       </c>
       <c r="I294" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e060:text</t>
+          <t>prism-brain-mapping:e069:text</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
@@ -12104,19 +12104,19 @@
       </c>
       <c r="D295" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E295" s="2" t="inlineStr">
         <is>
-          <t>Co pokazuje PRISM Brain Mapping?</t>
+          <t>PRISM może być wartościowym punktem wyjścia do rozwoju osobistego i zawodowego. Pomaga lepiej zrozumieć, dlaczego w jednych sytuacjach działamy spontanicznie i z łatwością, a inne wymagają od nas większego wysiłku. Badanie to może być również pomocne przy podejmowaniu decyzji dotyczących kariery, rozwoju kompetencji, komunikacji czy współpracy z innymi.</t>
         </is>
       </c>
       <c r="F295" s="4" t="inlineStr"/>
       <c r="G295" s="5" t="inlineStr"/>
       <c r="H295" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e060"]</t>
+          <t>p[data-content-id="e069"]</t>
         </is>
       </c>
       <c r="I295" s="2" t="inlineStr">
@@ -12128,7 +12128,7 @@
     <row r="296">
       <c r="A296" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e061:text</t>
+          <t>prism-brain-mapping:e070:text</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
@@ -12148,14 +12148,14 @@
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>Badanie odbywa się online i polega na udzieleniu odpowiedzi na kilkadziesiąt pytań. Na ich podstawie powstaje indywidualny profil przedstawiający 8 typów preferowanych zachowań oraz ich natężenie. PRISM pozwala również przyjrzeć się 26 czynnikom związanym z zachowaniem badanej osoby w określonych sytuacjach.</t>
+          <t>W przypadku organizacji PRISM znajduje zastosowanie między innymi w rozwoju liderów, budowaniu zespołów, rekrutacji, zarządzaniu talentami i planowaniu ścieżek rozwoju.</t>
         </is>
       </c>
       <c r="F296" s="4" t="inlineStr"/>
       <c r="G296" s="5" t="inlineStr"/>
       <c r="H296" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e061"]</t>
+          <t>p[data-content-id="e070"]</t>
         </is>
       </c>
       <c r="I296" s="2" t="inlineStr">
@@ -12167,7 +12167,7 @@
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e063:text</t>
+          <t>prism-brain-mapping:e071:text</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
@@ -12182,19 +12182,19 @@
       </c>
       <c r="D297" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E297" s="2" t="inlineStr">
         <is>
-          <t>Najbardziej charakterystycznym elementem badania jest mapa PRISM – przejrzysta wizualizacja, która pomaga zobaczyć własny profil psychologiczny z różnych perspektyw. Pokazuje między innymi naturalne preferencje zachowania, sposób, w jaki dostosowujemy się do wymagań otoczenia, oraz wzorzec zachowania, który najczęściej prezentujemy w relacjach z innymi.</t>
+          <t>Dlaczego warto omówić wynik z praktykiem?</t>
         </is>
       </c>
       <c r="F297" s="4" t="inlineStr"/>
       <c r="G297" s="5" t="inlineStr"/>
       <c r="H297" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e063"]</t>
+          <t>h2[data-content-id="e071"]</t>
         </is>
       </c>
       <c r="I297" s="2" t="inlineStr">
@@ -12206,7 +12206,7 @@
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e065:text</t>
+          <t>prism-brain-mapping:e072:text</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
@@ -12226,14 +12226,14 @@
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>PRISM dostarcza także informacji dotyczących inteligencji emocjonalnej, odporności psychicznej oraz cech osobowości w modelu Wielkiej Piątki. Dzięki temu pozwala szerzej spojrzeć na własne funkcjonowanie i dostrzec zarówno mocne strony, jak i obszary, które mogą wymagać większej uwagi.</t>
+          <t>Sam raport dostarcza wielu informacji, ale jego prawdziwa wartość zaczyna się, kiedy potrafimy odnieść go do własnej sytuacji. Podczas indywidualnej sesji wspólnie przyglądamy się Twojej mapie, interpretujemy poszczególne obszary i szukamy odpowiedzi na pytanie: co ta wiedza oznacza właśnie dla Ciebie?</t>
         </is>
       </c>
       <c r="F298" s="4" t="inlineStr"/>
       <c r="G298" s="5" t="inlineStr"/>
       <c r="H298" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e065"]</t>
+          <t>p[data-content-id="e072"]</t>
         </is>
       </c>
       <c r="I298" s="2" t="inlineStr">
@@ -12245,7 +12245,7 @@
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e068:text</t>
+          <t>prism-brain-mapping:e074:text</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
@@ -12260,19 +12260,19 @@
       </c>
       <c r="D299" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>Po co wykonywać PRISM Brain Mapping?</t>
+          <t>Rolą praktyka jest przełożenie wyników badania na język codziennych doświadczeń i konkretnych sytuacji – zawodowych, relacyjnych czy związanych z podejmowaniem decyzji. Dzięki temu PRISM nie pozostaje jedynie zestawem wyników, lecz może stać się punktem wyjścia do bardziej świadomego działania i rozwoju.</t>
         </is>
       </c>
       <c r="F299" s="4" t="inlineStr"/>
       <c r="G299" s="5" t="inlineStr"/>
       <c r="H299" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e068"]</t>
+          <t>p[data-content-id="e074"]</t>
         </is>
       </c>
       <c r="I299" s="2" t="inlineStr">
@@ -12284,7 +12284,7 @@
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e069:text</t>
+          <t>prism-brain-mapping:e075:text</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
@@ -12304,14 +12304,14 @@
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>PRISM może być wartościowym punktem wyjścia do rozwoju osobistego i zawodowego. Pomaga lepiej zrozumieć, dlaczego w jednych sytuacjach działamy spontanicznie i z łatwością, a inne wymagają od nas większego wysiłku. Badanie to może być również pomocne przy podejmowaniu decyzji dotyczących kariery, rozwoju kompetencji, komunikacji czy współpracy z innymi.</t>
+          <t>Jeśli chcesz lepiej poznać swoje naturalne preferencje i dowiedzieć się, jak świadomie wykorzystywać je w pracy i relacjach, zapraszam na badanie PRISM Brain Mapping wraz z indywidualną interpretacją wyników.</t>
         </is>
       </c>
       <c r="F300" s="4" t="inlineStr"/>
       <c r="G300" s="5" t="inlineStr"/>
       <c r="H300" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e069"]</t>
+          <t>p[data-content-id="e075"]</t>
         </is>
       </c>
       <c r="I300" s="2" t="inlineStr">
@@ -12323,7 +12323,7 @@
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e070:text</t>
+          <t>prism-brain-mapping:e078:href</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
@@ -12338,31 +12338,31 @@
       </c>
       <c r="D301" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E301" s="2" t="inlineStr">
         <is>
-          <t>W przypadku organizacji PRISM znajduje zastosowanie między innymi w rozwoju liderów, budowaniu zespołów, rekrutacji, zarządzaniu talentami i planowaniu ścieżek rozwoju.</t>
+          <t>index.html#kontakt</t>
         </is>
       </c>
       <c r="F301" s="4" t="inlineStr"/>
       <c r="G301" s="5" t="inlineStr"/>
       <c r="H301" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e070"]</t>
+          <t>a[data-content-id="e078"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I301" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e071:text</t>
+          <t>prism-brain-mapping:e078:text</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
@@ -12377,19 +12377,19 @@
       </c>
       <c r="D302" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
-          <t>Dlaczego warto omówić wynik z praktykiem?</t>
+          <t>Umów konsultację</t>
         </is>
       </c>
       <c r="F302" s="4" t="inlineStr"/>
       <c r="G302" s="5" t="inlineStr"/>
       <c r="H302" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e071"]</t>
+          <t>a[data-content-id="e078"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I302" s="2" t="inlineStr">
@@ -12401,73 +12401,73 @@
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e072:text</t>
+          <t>mtq-plus:e006:content</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping.html</t>
+          <t>mtq-plus.html</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>PRISM Brain Mapping</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Opis strony (meta description)</t>
         </is>
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>Sam raport dostarcza wielu informacji, ale jego prawdziwa wartość zaczyna się, kiedy potrafimy odnieść go do własnej sytuacji. Podczas indywidualnej sesji wspólnie przyglądamy się Twojej mapie, interpretujemy poszczególne obszary i szukamy odpowiedzi na pytanie: co ta wiedza oznacza właśnie dla Ciebie?</t>
+          <t>MTQ Plus. Diagnoza i rozwój inteligencji mentalnej, odporności psychicznej i zasobów wewnętrznych.</t>
         </is>
       </c>
       <c r="F303" s="4" t="inlineStr"/>
       <c r="G303" s="5" t="inlineStr"/>
       <c r="H303" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e072"]</t>
+          <t>meta[data-content-id="e006"]</t>
         </is>
       </c>
       <c r="I303" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>content</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e074:text</t>
+          <t>mtq-plus:e007:text</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping.html</t>
+          <t>mtq-plus.html</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>PRISM Brain Mapping</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Tytuł strony</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>Rolą praktyka jest przełożenie wyników badania na język codziennych doświadczeń i konkretnych sytuacji – zawodowych, relacyjnych czy związanych z podejmowaniem decyzji. Dzięki temu PRISM nie pozostaje jedynie zestawem wyników, lecz może stać się punktem wyjścia do bardziej świadomego działania i rozwoju.</t>
+          <t>MTQ Plus — Katarzyna Chałas</t>
         </is>
       </c>
       <c r="F304" s="4" t="inlineStr"/>
       <c r="G304" s="5" t="inlineStr"/>
       <c r="H304" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e074"]</t>
+          <t>title[data-content-id="e007"]</t>
         </is>
       </c>
       <c r="I304" s="2" t="inlineStr">
@@ -12479,124 +12479,124 @@
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e075:text</t>
+          <t>mtq-plus:e015:href</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping.html</t>
+          <t>mtq-plus.html</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>PRISM Brain Mapping</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>Jeśli chcesz lepiej poznać swoje naturalne preferencje i dowiedzieć się, jak świadomie wykorzystywać je w pracy i relacjach, zapraszam na badanie PRISM Brain Mapping wraz z indywidualną interpretacją wyników.</t>
+          <t>#main-content</t>
         </is>
       </c>
       <c r="F305" s="4" t="inlineStr"/>
       <c r="G305" s="5" t="inlineStr"/>
       <c r="H305" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e075"]</t>
+          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
         </is>
       </c>
       <c r="I305" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e078:href</t>
+          <t>mtq-plus:e015:text</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping.html</t>
+          <t>mtq-plus.html</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>PRISM Brain Mapping</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
-          <t>index.html#kontakt</t>
+          <t>Przejdź do treści</t>
         </is>
       </c>
       <c r="F306" s="4" t="inlineStr"/>
       <c r="G306" s="5" t="inlineStr"/>
       <c r="H306" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e078"] | Umów konsultację → index.html#kontakt</t>
+          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
         </is>
       </c>
       <c r="I306" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping:e078:text</t>
+          <t>mtq-plus:e042:href</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>prism-brain-mapping.html</t>
+          <t>mtq-plus.html</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>PRISM Brain Mapping</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E307" s="2" t="inlineStr">
         <is>
-          <t>Umów konsultację</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="F307" s="4" t="inlineStr"/>
       <c r="G307" s="5" t="inlineStr"/>
       <c r="H307" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e078"] | Umów konsultację → index.html#kontakt</t>
+          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
         </is>
       </c>
       <c r="I307" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e006:content</t>
+          <t>mtq-plus:e042:text</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
@@ -12606,36 +12606,36 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>Opis strony (meta description)</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus. Diagnoza i rozwój inteligencji mentalnej, odporności psychicznej i zasobów wewnętrznych.</t>
+          <t>← Strona główna</t>
         </is>
       </c>
       <c r="F308" s="4" t="inlineStr"/>
       <c r="G308" s="5" t="inlineStr"/>
       <c r="H308" s="2" t="inlineStr">
         <is>
-          <t>meta[data-content-id="e006"]</t>
+          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
         </is>
       </c>
       <c r="I308" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e007:text</t>
+          <t>mtq-plus:e043:text</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
@@ -12645,24 +12645,24 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>Tytuł strony</t>
+          <t>Nagłówek H1</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus — Katarzyna Chałas</t>
+          <t>MTQ Plus</t>
         </is>
       </c>
       <c r="F309" s="4" t="inlineStr"/>
       <c r="G309" s="5" t="inlineStr"/>
       <c r="H309" s="2" t="inlineStr">
         <is>
-          <t>title[data-content-id="e007"]</t>
+          <t>h1[data-content-id="e043"]</t>
         </is>
       </c>
       <c r="I309" s="2" t="inlineStr">
@@ -12674,7 +12674,7 @@
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e015:href</t>
+          <t>mtq-plus:e044:text</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
@@ -12684,36 +12684,36 @@
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>#main-content</t>
+          <t>Diagnoza i rozwój inteligencji mentalnej, odporności psychicznej i zasobów wewnętrznych.</t>
         </is>
       </c>
       <c r="F310" s="4" t="inlineStr"/>
       <c r="G310" s="5" t="inlineStr"/>
       <c r="H310" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
+          <t>p[data-content-id="e044"]</t>
         </is>
       </c>
       <c r="I310" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e015:text</t>
+          <t>mtq-plus:e046:alt</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
@@ -12723,36 +12723,36 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Opis obrazu (alt)</t>
         </is>
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
-          <t>Przejdź do treści</t>
+          <t>Logo badania MTQ Plus</t>
         </is>
       </c>
       <c r="F311" s="4" t="inlineStr"/>
       <c r="G311" s="5" t="inlineStr"/>
       <c r="H311" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
+          <t>img[data-content-id="e046"] | assets/hero-mtq-plus.webp</t>
         </is>
       </c>
       <c r="I311" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>alt</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e042:href</t>
+          <t>mtq-plus:e049:text</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
@@ -12762,36 +12762,36 @@
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>MTQ Plus</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>index.html</t>
+          <t>Od kilku lat przeprowadzam i omawiam badania MTQ Plus – pierwszego na świecie narzędzia do pomiaru odporności psychicznej. Wraz z raportem obejmującym wyniki testu, osoby i organizacje, które wspieram, otrzymują indywidualny plan rozwojowy. Jest to badanie szczególnie przydatne w procesie coachingowym i często zalecam je jako punkt wyjścia do dalszego rozwoju.</t>
         </is>
       </c>
       <c r="F312" s="4" t="inlineStr"/>
       <c r="G312" s="5" t="inlineStr"/>
       <c r="H312" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>p[data-content-id="e049"]</t>
         </is>
       </c>
       <c r="I312" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e042:text</t>
+          <t>mtq-plus:e050:text</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
@@ -12801,24 +12801,24 @@
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>MTQ Plus</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Czym jest badanie MTQ Plus?</t>
         </is>
       </c>
       <c r="F313" s="4" t="inlineStr"/>
       <c r="G313" s="5" t="inlineStr"/>
       <c r="H313" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>h2[data-content-id="e050"]</t>
         </is>
       </c>
       <c r="I313" s="2" t="inlineStr">
@@ -12830,7 +12830,7 @@
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e043:text</t>
+          <t>mtq-plus:e051:text</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
@@ -12840,24 +12840,24 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>MTQ Plus</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H1</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus</t>
+          <t>Czy chcesz dowiedzieć się, jak tak naprawdę się zachowujesz, gdy rośnie presja, pojawia się niepewność albo coś nie idzie zgodnie z planem? Czy potrafisz zachować spokój i wpływać na bieg wydarzeń? Jak podchodzisz do ambitnych celów, ryzyka i niepowodzeń? I co dzieje się z Twoją pewnością siebie, gdy sytuacja stawia Cię przed trudnym zadaniem?</t>
         </is>
       </c>
       <c r="F314" s="4" t="inlineStr"/>
       <c r="G314" s="5" t="inlineStr"/>
       <c r="H314" s="2" t="inlineStr">
         <is>
-          <t>h1[data-content-id="e043"]</t>
+          <t>p[data-content-id="e051"]</t>
         </is>
       </c>
       <c r="I314" s="2" t="inlineStr">
@@ -12869,7 +12869,7 @@
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e044:text</t>
+          <t>mtq-plus:e052:text</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
@@ -12879,7 +12879,7 @@
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>MTQ Plus</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
@@ -12889,14 +12889,14 @@
       </c>
       <c r="E315" s="2" t="inlineStr">
         <is>
-          <t>Diagnoza i rozwój inteligencji mentalnej, odporności psychicznej i zasobów wewnętrznych.</t>
+          <t>MTQ Plus to profesjonalne narzędzie psychometryczne, które pomaga lepiej zrozumieć sposób, w jaki myślisz i reagujesz w obliczu presji, stresu, zmian i wyzwań. Pokazuje Twój indywidualny profil mental toughness – obszary, które są Twoimi zasobami, oraz te, które mogą wymagać większej uwagi i świadomego rozwoju.</t>
         </is>
       </c>
       <c r="F315" s="4" t="inlineStr"/>
       <c r="G315" s="5" t="inlineStr"/>
       <c r="H315" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e044"]</t>
+          <t>p[data-content-id="e052"]</t>
         </is>
       </c>
       <c r="I315" s="2" t="inlineStr">
@@ -12908,7 +12908,7 @@
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e046:alt</t>
+          <t>mtq-plus:e054:text</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
@@ -12918,36 +12918,36 @@
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>MTQ Plus</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
         <is>
-          <t>Opis obrazu (alt)</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E316" s="2" t="inlineStr">
         <is>
-          <t>Logo badania MTQ Plus</t>
+          <t>Co bada MTQ Plus?</t>
         </is>
       </c>
       <c r="F316" s="4" t="inlineStr"/>
       <c r="G316" s="5" t="inlineStr"/>
       <c r="H316" s="2" t="inlineStr">
         <is>
-          <t>img[data-content-id="e046"] | assets/hero-mtq-plus.webp</t>
+          <t>h2[data-content-id="e054"]</t>
         </is>
       </c>
       <c r="I316" s="2" t="inlineStr">
         <is>
-          <t>alt</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e049:text</t>
+          <t>mtq-plus:e055:text</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
@@ -12967,14 +12967,14 @@
       </c>
       <c r="E317" s="2" t="inlineStr">
         <is>
-          <t>Od kilku lat przeprowadzam i omawiam badania MTQ Plus – pierwszego na świecie narzędzia do pomiaru odporności psychicznej. Wraz z raportem obejmującym wyniki testu, osoby i organizacje, które wspieram, otrzymują indywidualny plan rozwojowy. Jest to badanie szczególnie przydatne w procesie coachingowym i często zalecam je jako punkt wyjścia do dalszego rozwoju.</t>
+          <t>Model MTQ Plus opiera się na czterech obszarach: Control (poczucie kontroli), Commitment (zaangażowanie), Challenge (wyzwanie) i Confidence (pewność siebie). Każdy z nich dzieli się na dwa bardziej szczegółowe wymiary:</t>
         </is>
       </c>
       <c r="F317" s="4" t="inlineStr"/>
       <c r="G317" s="5" t="inlineStr"/>
       <c r="H317" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e049"]</t>
+          <t>p[data-content-id="e055"]</t>
         </is>
       </c>
       <c r="I317" s="2" t="inlineStr">
@@ -12986,7 +12986,7 @@
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e050:text</t>
+          <t>mtq-plus:e061:text</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
@@ -13001,19 +13001,19 @@
       </c>
       <c r="D318" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Punkt listy</t>
         </is>
       </c>
       <c r="E318" s="2" t="inlineStr">
         <is>
-          <t>Czym jest badanie MTQ Plus?</t>
+          <t>kontrola à poczucie wpływu na własne życie + umiejętność zarządzania emocjami</t>
         </is>
       </c>
       <c r="F318" s="4" t="inlineStr"/>
       <c r="G318" s="5" t="inlineStr"/>
       <c r="H318" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e050"]</t>
+          <t>li[data-content-id="e061"]</t>
         </is>
       </c>
       <c r="I318" s="2" t="inlineStr">
@@ -13025,7 +13025,7 @@
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e051:text</t>
+          <t>mtq-plus:e062:text</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
@@ -13040,19 +13040,19 @@
       </c>
       <c r="D319" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Punkt listy</t>
         </is>
       </c>
       <c r="E319" s="2" t="inlineStr">
         <is>
-          <t>Czy chcesz dowiedzieć się, jak tak naprawdę się zachowujesz, gdy rośnie presja, pojawia się niepewność albo coś nie idzie zgodnie z planem? Czy potrafisz zachować spokój i wpływać na bieg wydarzeń? Jak podchodzisz do ambitnych celów, ryzyka i niepowodzeń? I co dzieje się z Twoją pewnością siebie, gdy sytuacja stawia Cię przed trudnym zadaniem?</t>
+          <t>zaangażowanie à orientacja na cele + gotowość do podejmowania wysiłku potrzebnego do ich realizacji</t>
         </is>
       </c>
       <c r="F319" s="4" t="inlineStr"/>
       <c r="G319" s="5" t="inlineStr"/>
       <c r="H319" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e051"]</t>
+          <t>li[data-content-id="e062"]</t>
         </is>
       </c>
       <c r="I319" s="2" t="inlineStr">
@@ -13064,7 +13064,7 @@
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e052:text</t>
+          <t>mtq-plus:e063:text</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
@@ -13079,19 +13079,19 @@
       </c>
       <c r="D320" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Punkt listy</t>
         </is>
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus to profesjonalne narzędzie psychometryczne, które pomaga lepiej zrozumieć sposób, w jaki myślisz i reagujesz w obliczu presji, stresu, zmian i wyzwań. Pokazuje Twój indywidualny profil mental toughness – obszary, które są Twoimi zasobami, oraz te, które mogą wymagać większej uwagi i świadomego rozwoju.</t>
+          <t>wyzwanie à stosunek do ryzyka + zdolność do wyciągania wniosków z doświadczeń i niepowodzeń</t>
         </is>
       </c>
       <c r="F320" s="4" t="inlineStr"/>
       <c r="G320" s="5" t="inlineStr"/>
       <c r="H320" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e052"]</t>
+          <t>li[data-content-id="e063"]</t>
         </is>
       </c>
       <c r="I320" s="2" t="inlineStr">
@@ -13103,7 +13103,7 @@
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e054:text</t>
+          <t>mtq-plus:e064:text</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">
@@ -13118,19 +13118,19 @@
       </c>
       <c r="D321" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Punkt listy</t>
         </is>
       </c>
       <c r="E321" s="2" t="inlineStr">
         <is>
-          <t>Co bada MTQ Plus?</t>
+          <t>pewność siebie à wiara we własne możliwości + swoboda w relacjach z innymi</t>
         </is>
       </c>
       <c r="F321" s="4" t="inlineStr"/>
       <c r="G321" s="5" t="inlineStr"/>
       <c r="H321" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e054"]</t>
+          <t>li[data-content-id="e064"]</t>
         </is>
       </c>
       <c r="I321" s="2" t="inlineStr">
@@ -13142,7 +13142,7 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e055:text</t>
+          <t>mtq-plus:e065:text</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
@@ -13162,14 +13162,14 @@
       </c>
       <c r="E322" s="2" t="inlineStr">
         <is>
-          <t>Model MTQ Plus opiera się na czterech obszarach: Control (poczucie kontroli), Commitment (zaangażowanie), Challenge (wyzwanie) i Confidence (pewność siebie). Każdy z nich dzieli się na dwa bardziej szczegółowe wymiary:</t>
+          <t>To narzędzie psychometryczne pozwala więc spojrzeć na siebie szerzej niż przez pryzmat pojedynczej cechy. Dwie osoby mogą podobnie radzić sobie z presją, ale osiągać ten efekt w zupełnie inny sposób. Właśnie dlatego istotny jest nie tylko wynik ogólny, lecz przede wszystkim indywidualny układ poszczególnych obszarów.</t>
         </is>
       </c>
       <c r="F322" s="4" t="inlineStr"/>
       <c r="G322" s="5" t="inlineStr"/>
       <c r="H322" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e055"]</t>
+          <t>p[data-content-id="e065"]</t>
         </is>
       </c>
       <c r="I322" s="2" t="inlineStr">
@@ -13181,7 +13181,7 @@
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e061:text</t>
+          <t>mtq-plus:e067:text</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
@@ -13196,19 +13196,19 @@
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>Punkt listy</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E323" s="2" t="inlineStr">
         <is>
-          <t>kontrola à poczucie wpływu na własne życie + umiejętność zarządzania emocjami</t>
+          <t>Po co wykonywać test MTQ Plus?</t>
         </is>
       </c>
       <c r="F323" s="4" t="inlineStr"/>
       <c r="G323" s="5" t="inlineStr"/>
       <c r="H323" s="2" t="inlineStr">
         <is>
-          <t>li[data-content-id="e061"]</t>
+          <t>h2[data-content-id="e067"]</t>
         </is>
       </c>
       <c r="I323" s="2" t="inlineStr">
@@ -13220,7 +13220,7 @@
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e062:text</t>
+          <t>mtq-plus:e068:text</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
@@ -13235,19 +13235,19 @@
       </c>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>Punkt listy</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr">
         <is>
-          <t>zaangażowanie à orientacja na cele + gotowość do podejmowania wysiłku potrzebnego do ich realizacji</t>
+          <t>Wynik testu może stać się punktem wyjścia do bardziej świadomego rozwoju – zarówno zawodowego, jak i osobistego. Pomaga nazwać mechanizmy, które wcześniej mogły być trudne do zauważenia, lepiej zrozumieć własne reakcje i określić, nad czym warto pracować.</t>
         </is>
       </c>
       <c r="F324" s="4" t="inlineStr"/>
       <c r="G324" s="5" t="inlineStr"/>
       <c r="H324" s="2" t="inlineStr">
         <is>
-          <t>li[data-content-id="e062"]</t>
+          <t>p[data-content-id="e068"]</t>
         </is>
       </c>
       <c r="I324" s="2" t="inlineStr">
@@ -13259,7 +13259,7 @@
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e063:text</t>
+          <t>mtq-plus:e069:text</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
@@ -13274,19 +13274,19 @@
       </c>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>Punkt listy</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr">
         <is>
-          <t>wyzwanie à stosunek do ryzyka + zdolność do wyciągania wniosków z doświadczeń i niepowodzeń</t>
+          <t>Szczególnie wartościowe jest połączenie samego badania z profesjonalną interpretacją. Raport dostarcza danych, ale dopiero rozmowa pozwala odnieść je do Twojej rzeczywistości: pracy, relacji, podejmowania decyzji czy sytuacji, w których odczuwasz szczególną presję.</t>
         </is>
       </c>
       <c r="F325" s="4" t="inlineStr"/>
       <c r="G325" s="5" t="inlineStr"/>
       <c r="H325" s="2" t="inlineStr">
         <is>
-          <t>li[data-content-id="e063"]</t>
+          <t>p[data-content-id="e069"]</t>
         </is>
       </c>
       <c r="I325" s="2" t="inlineStr">
@@ -13298,7 +13298,7 @@
     <row r="326">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e064:text</t>
+          <t>mtq-plus:e070:text</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
@@ -13313,19 +13313,19 @@
       </c>
       <c r="D326" s="2" t="inlineStr">
         <is>
-          <t>Punkt listy</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E326" s="2" t="inlineStr">
         <is>
-          <t>pewność siebie à wiara we własne możliwości + swoboda w relacjach z innymi</t>
+          <t>Test MTQ Plus wykonuję wraz z indywidualną interpretacją wyników, tak aby badanie nie kończyło się na wykresie i liczbach. Wspólnie przyglądamy się Twojemu profilowi, jego mocnym stronom i obszarom rozwoju, a następnie przekładamy wnioski na praktyczne działania.</t>
         </is>
       </c>
       <c r="F326" s="4" t="inlineStr"/>
       <c r="G326" s="5" t="inlineStr"/>
       <c r="H326" s="2" t="inlineStr">
         <is>
-          <t>li[data-content-id="e064"]</t>
+          <t>p[data-content-id="e070"]</t>
         </is>
       </c>
       <c r="I326" s="2" t="inlineStr">
@@ -13337,7 +13337,7 @@
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e065:text</t>
+          <t>mtq-plus:e072:text</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
@@ -13357,14 +13357,14 @@
       </c>
       <c r="E327" s="2" t="inlineStr">
         <is>
-          <t>To narzędzie psychometryczne pozwala więc spojrzeć na siebie szerzej niż przez pryzmat pojedynczej cechy. Dwie osoby mogą podobnie radzić sobie z presją, ale osiągać ten efekt w zupełnie inny sposób. Właśnie dlatego istotny jest nie tylko wynik ogólny, lecz przede wszystkim indywidualny układ poszczególnych obszarów.</t>
+          <t>Jeśli chcesz lepiej rozumieć siebie, skuteczniej wykorzystywać swoje zasoby i świadomie rozwijać sposób, w jaki reagujesz na wyzwania, MTQ Plus może być dobrym początkiem.</t>
         </is>
       </c>
       <c r="F327" s="4" t="inlineStr"/>
       <c r="G327" s="5" t="inlineStr"/>
       <c r="H327" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e065"]</t>
+          <t>p[data-content-id="e072"]</t>
         </is>
       </c>
       <c r="I327" s="2" t="inlineStr">
@@ -13376,7 +13376,7 @@
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e067:text</t>
+          <t>mtq-plus:e075:href</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
@@ -13391,31 +13391,31 @@
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>Po co wykonywać test MTQ Plus?</t>
+          <t>index.html#kontakt</t>
         </is>
       </c>
       <c r="F328" s="4" t="inlineStr"/>
       <c r="G328" s="5" t="inlineStr"/>
       <c r="H328" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e067"]</t>
+          <t>a[data-content-id="e075"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I328" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e068:text</t>
+          <t>mtq-plus:e075:text</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
@@ -13430,19 +13430,19 @@
       </c>
       <c r="D329" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E329" s="2" t="inlineStr">
         <is>
-          <t>Wynik testu może stać się punktem wyjścia do bardziej świadomego rozwoju – zarówno zawodowego, jak i osobistego. Pomaga nazwać mechanizmy, które wcześniej mogły być trudne do zauważenia, lepiej zrozumieć własne reakcje i określić, nad czym warto pracować.</t>
+          <t>Umów konsultację</t>
         </is>
       </c>
       <c r="F329" s="4" t="inlineStr"/>
       <c r="G329" s="5" t="inlineStr"/>
       <c r="H329" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e068"]</t>
+          <t>a[data-content-id="e075"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I329" s="2" t="inlineStr">
@@ -13454,73 +13454,73 @@
     <row r="330">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e069:text</t>
+          <t>terapia-dzwiekiem:e006:content</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus.html</t>
+          <t>terapia-dzwiekiem.html</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Opis strony (meta description)</t>
         </is>
       </c>
       <c r="E330" s="2" t="inlineStr">
         <is>
-          <t>Szczególnie wartościowe jest połączenie samego badania z profesjonalną interpretacją. Raport dostarcza danych, ale dopiero rozmowa pozwala odnieść je do Twojej rzeczywistości: pracy, relacji, podejmowania decyzji czy sytuacji, w których odczuwasz szczególną presję.</t>
+          <t>Terapia dźwiękiem. Praca z dźwiękiem dla redukcji stresu, regeneracji układu nerwowego i osiągnięcia harmonii ciała oraz umysłu</t>
         </is>
       </c>
       <c r="F330" s="4" t="inlineStr"/>
       <c r="G330" s="5" t="inlineStr"/>
       <c r="H330" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e069"]</t>
+          <t>meta[data-content-id="e006"]</t>
         </is>
       </c>
       <c r="I330" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>content</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e070:text</t>
+          <t>terapia-dzwiekiem:e007:text</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus.html</t>
+          <t>terapia-dzwiekiem.html</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Tytuł strony</t>
         </is>
       </c>
       <c r="E331" s="2" t="inlineStr">
         <is>
-          <t>Test MTQ Plus wykonuję wraz z indywidualną interpretacją wyników, tak aby badanie nie kończyło się na wykresie i liczbach. Wspólnie przyglądamy się Twojemu profilowi, jego mocnym stronom i obszarom rozwoju, a następnie przekładamy wnioski na praktyczne działania.</t>
+          <t>Terapia dźwiękiem — Katarzyna Chałas</t>
         </is>
       </c>
       <c r="F331" s="4" t="inlineStr"/>
       <c r="G331" s="5" t="inlineStr"/>
       <c r="H331" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e070"]</t>
+          <t>title[data-content-id="e007"]</t>
         </is>
       </c>
       <c r="I331" s="2" t="inlineStr">
@@ -13532,124 +13532,124 @@
     <row r="332">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e072:text</t>
+          <t>terapia-dzwiekiem:e015:href</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus.html</t>
+          <t>terapia-dzwiekiem.html</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E332" s="2" t="inlineStr">
         <is>
-          <t>Jeśli chcesz lepiej rozumieć siebie, skuteczniej wykorzystywać swoje zasoby i świadomie rozwijać sposób, w jaki reagujesz na wyzwania, MTQ Plus może być dobrym początkiem.</t>
+          <t>#main-content</t>
         </is>
       </c>
       <c r="F332" s="4" t="inlineStr"/>
       <c r="G332" s="5" t="inlineStr"/>
       <c r="H332" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e072"]</t>
+          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
         </is>
       </c>
       <c r="I332" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e075:href</t>
+          <t>terapia-dzwiekiem:e015:text</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus.html</t>
+          <t>terapia-dzwiekiem.html</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E333" s="2" t="inlineStr">
         <is>
-          <t>index.html#kontakt</t>
+          <t>Przejdź do treści</t>
         </is>
       </c>
       <c r="F333" s="4" t="inlineStr"/>
       <c r="G333" s="5" t="inlineStr"/>
       <c r="H333" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e075"] | Umów konsultację → index.html#kontakt</t>
+          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
         </is>
       </c>
       <c r="I333" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus:e075:text</t>
+          <t>terapia-dzwiekiem:e042:href</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>mtq-plus.html</t>
+          <t>terapia-dzwiekiem.html</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>MTQ Plus</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E334" s="2" t="inlineStr">
         <is>
-          <t>Umów konsultację</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="F334" s="4" t="inlineStr"/>
       <c r="G334" s="5" t="inlineStr"/>
       <c r="H334" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e075"] | Umów konsultację → index.html#kontakt</t>
+          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
         </is>
       </c>
       <c r="I334" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e006:content</t>
+          <t>terapia-dzwiekiem:e042:text</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
@@ -13659,36 +13659,36 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D335" s="2" t="inlineStr">
         <is>
-          <t>Opis strony (meta description)</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E335" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem. Praca z dźwiękiem dla redukcji stresu, regeneracji układu nerwowego i osiągnięcia harmonii ciała oraz umysłu</t>
+          <t>← Strona główna</t>
         </is>
       </c>
       <c r="F335" s="4" t="inlineStr"/>
       <c r="G335" s="5" t="inlineStr"/>
       <c r="H335" s="2" t="inlineStr">
         <is>
-          <t>meta[data-content-id="e006"]</t>
+          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
         </is>
       </c>
       <c r="I335" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e007:text</t>
+          <t>terapia-dzwiekiem:e043:text</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
@@ -13698,24 +13698,24 @@
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
         <is>
-          <t>Tytuł strony</t>
+          <t>Nagłówek H1</t>
         </is>
       </c>
       <c r="E336" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem — Katarzyna Chałas</t>
+          <t>Terapia dźwiękiem</t>
         </is>
       </c>
       <c r="F336" s="4" t="inlineStr"/>
       <c r="G336" s="5" t="inlineStr"/>
       <c r="H336" s="2" t="inlineStr">
         <is>
-          <t>title[data-content-id="e007"]</t>
+          <t>h1[data-content-id="e043"]</t>
         </is>
       </c>
       <c r="I336" s="2" t="inlineStr">
@@ -13727,7 +13727,7 @@
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e015:href</t>
+          <t>terapia-dzwiekiem:e044:text</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
@@ -13737,36 +13737,36 @@
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
         <is>
-          <t>#main-content</t>
+          <t>Praca z dźwiękiem dla redukcji stresu, regeneracji układu nerwowego i osiągnięcia harmonii ciała oraz umysłu</t>
         </is>
       </c>
       <c r="F337" s="4" t="inlineStr"/>
       <c r="G337" s="5" t="inlineStr"/>
       <c r="H337" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
+          <t>p[data-content-id="e044"]</t>
         </is>
       </c>
       <c r="I337" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e015:text</t>
+          <t>terapia-dzwiekiem:e046:alt</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
@@ -13776,36 +13776,36 @@
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Opis obrazu (alt)</t>
         </is>
       </c>
       <c r="E338" s="2" t="inlineStr">
         <is>
-          <t>Przejdź do treści</t>
+          <t>Katarzyna Chałas z misami dźwiękowymi</t>
         </is>
       </c>
       <c r="F338" s="4" t="inlineStr"/>
       <c r="G338" s="5" t="inlineStr"/>
       <c r="H338" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
+          <t>img[data-content-id="e046"] | assets/hero-terapia-1000.webp</t>
         </is>
       </c>
       <c r="I338" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>alt</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e042:href</t>
+          <t>terapia-dzwiekiem:e049:text</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
@@ -13815,36 +13815,36 @@
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Terapia dźwiękiem</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E339" s="2" t="inlineStr">
         <is>
-          <t>index.html</t>
+          <t>Uzupełnieniem mojej pracy na polu poznawczym i doradczym jest praca z ciałem poprzez dźwięk i wibracje. Masaż dźwiękiem metodą Petera Hessa®, którego jestem certyfikowaną praktyczką, wspomaga regulację układu nerwowego, regenerację organizmu i redukcję napięcia. Zapraszam do bezpiecznej, spokojnej przestrzeni, w której na nowo nawiążesz kontakt z ciałem, co jest szczególnie ważne u osób przeciążonych stresem, presją i odpowiedzialnością.</t>
         </is>
       </c>
       <c r="F339" s="4" t="inlineStr"/>
       <c r="G339" s="5" t="inlineStr"/>
       <c r="H339" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>p[data-content-id="e049"]</t>
         </is>
       </c>
       <c r="I339" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e042:text</t>
+          <t>terapia-dzwiekiem:e050:text</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
@@ -13854,24 +13854,24 @@
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Terapia dźwiękiem</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Na czym polega masaż dźwiękiem Metodą Petera Hessa®?</t>
         </is>
       </c>
       <c r="F340" s="4" t="inlineStr"/>
       <c r="G340" s="5" t="inlineStr"/>
       <c r="H340" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>h2[data-content-id="e050"]</t>
         </is>
       </c>
       <c r="I340" s="2" t="inlineStr">
@@ -13883,7 +13883,7 @@
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e043:text</t>
+          <t>terapia-dzwiekiem:e051:text</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
@@ -13893,24 +13893,24 @@
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Terapia dźwiękiem</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H1</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem</t>
+          <t>Podczas sesji na ciele układane są specjalne misy dźwiękowe, które następnie pobudzam do wibracji za pomocą filcowej pałeczki. Dzięki temu dźwięk i delikatne drgania są odbierane nie tylko przez słuch, lecz także przez ciało.</t>
         </is>
       </c>
       <c r="F341" s="4" t="inlineStr"/>
       <c r="G341" s="5" t="inlineStr"/>
       <c r="H341" s="2" t="inlineStr">
         <is>
-          <t>h1[data-content-id="e043"]</t>
+          <t>p[data-content-id="e051"]</t>
         </is>
       </c>
       <c r="I341" s="2" t="inlineStr">
@@ -13922,7 +13922,7 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e044:text</t>
+          <t>terapia-dzwiekiem:e052:text</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
@@ -13932,7 +13932,7 @@
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Terapia dźwiękiem</t>
         </is>
       </c>
       <c r="D342" s="2" t="inlineStr">
@@ -13942,14 +13942,14 @@
       </c>
       <c r="E342" s="2" t="inlineStr">
         <is>
-          <t>Praca z dźwiękiem dla redukcji stresu, regeneracji układu nerwowego i osiągnięcia harmonii ciała oraz umysłu</t>
+          <t>Sesja odbywa się w pozycji leżącej, w ubraniu, które nie krępuje ruchów. Misy mogą być układane w różnych obszarach ciała, między innymi w okolicy stóp, pleców, lędźwi, klatki piersiowej, ramion czy dłoni. Poszczególne elementy masażu dobieram z uwzględnieniem Twoich potrzeb i możliwości. Metoda Petera Hessa® opiera się nie tylko na określonej technice pracy z misami, lecz także na uważności i indywidualnym podejściu do osoby, która z niej korzysta.</t>
         </is>
       </c>
       <c r="F342" s="4" t="inlineStr"/>
       <c r="G342" s="5" t="inlineStr"/>
       <c r="H342" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e044"]</t>
+          <t>p[data-content-id="e052"]</t>
         </is>
       </c>
       <c r="I342" s="2" t="inlineStr">
@@ -13961,7 +13961,7 @@
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e046:alt</t>
+          <t>terapia-dzwiekiem:e053:text</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
@@ -13971,36 +13971,36 @@
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Terapia dźwiękiem</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
         <is>
-          <t>Opis obrazu (alt)</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E343" s="2" t="inlineStr">
         <is>
-          <t>Katarzyna Chałas z misami dźwiękowymi</t>
+          <t>Dźwięki kolejnych mis tworzą harmonię, dzięki której łatwiej zwolnić tempo i skierować uwagę do wewnątrz. Dla wielu osób jest to doświadczenie głębokiego relaksu, pozwalające choć na chwilę odłączyć się od codziennego natłoku myśli i bodźców.</t>
         </is>
       </c>
       <c r="F343" s="4" t="inlineStr"/>
       <c r="G343" s="5" t="inlineStr"/>
       <c r="H343" s="2" t="inlineStr">
         <is>
-          <t>img[data-content-id="e046"] | assets/hero-terapia-1000.webp</t>
+          <t>p[data-content-id="e053"]</t>
         </is>
       </c>
       <c r="I343" s="2" t="inlineStr">
         <is>
-          <t>alt</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e049:text</t>
+          <t>terapia-dzwiekiem:e054:text</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
@@ -14015,19 +14015,19 @@
       </c>
       <c r="D344" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E344" s="2" t="inlineStr">
         <is>
-          <t>Uzupełnieniem mojej pracy na polu poznawczym i doradczym jest praca z ciałem poprzez dźwięk i wibracje. Masaż dźwiękiem metodą Petera Hessa®, którego jestem certyfikowaną praktyczką, wspomaga regulację układu nerwowego, regenerację organizmu i redukcję napięcia. Zapraszam do bezpiecznej, spokojnej przestrzeni, w której na nowo nawiążesz kontakt z ciałem, co jest szczególnie ważne u osób przeciążonych stresem, presją i odpowiedzialnością.</t>
+          <t>Dlaczego wybrałam Metodę Petera Hessa®?</t>
         </is>
       </c>
       <c r="F344" s="4" t="inlineStr"/>
       <c r="G344" s="5" t="inlineStr"/>
       <c r="H344" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e049"]</t>
+          <t>h2[data-content-id="e054"]</t>
         </is>
       </c>
       <c r="I344" s="2" t="inlineStr">
@@ -14039,7 +14039,7 @@
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e050:text</t>
+          <t>terapia-dzwiekiem:e055:text</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
@@ -14054,19 +14054,19 @@
       </c>
       <c r="D345" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E345" s="2" t="inlineStr">
         <is>
-          <t>Na czym polega masaż dźwiękiem Metodą Petera Hessa®?</t>
+          <t>Została ona opracowana przez niemieckiego fizyka Petera Hessa na początku lat 80. XX wieku i jest do dziś szeroko wykorzystywana m.in. w obszarze relaksacji, odnowy biologicznej, pedagogiki i pracy wspierającej. Jej ważnym elementem jest indywidualne podejście – sposób prowadzenia masażu może być dostosowany do konkretnej osoby, jej aktualnych potrzeb i możliwości, z uwzględnieniem znajomości fizjologii i biologii ludzkiego ciała.</t>
         </is>
       </c>
       <c r="F345" s="4" t="inlineStr"/>
       <c r="G345" s="5" t="inlineStr"/>
       <c r="H345" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e050"]</t>
+          <t>p[data-content-id="e055"]</t>
         </is>
       </c>
       <c r="I345" s="2" t="inlineStr">
@@ -14078,7 +14078,7 @@
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e051:text</t>
+          <t>terapia-dzwiekiem:e056:text</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
@@ -14098,14 +14098,14 @@
       </c>
       <c r="E346" s="2" t="inlineStr">
         <is>
-          <t>Podczas sesji na ciele układane są specjalne misy dźwiękowe, które następnie pobudzam do wibracji za pomocą filcowej pałeczki. Dzięki temu dźwięk i delikatne drgania są odbierane nie tylko przez słuch, lecz także przez ciało.</t>
+          <t>Metoda ta jest sprawdzona i godna zaufania jako technika relaksacyjna. Nie jest zbiorem sztywnych procedur, ale pozwala na dopasowanie przebiegu spotkania do potrzeb danej osoby i na czerpanie radości z obserwacji, jak wzrasta spokój i harmonia. A wreszcie – jest nieustannym kontaktem z pięknem muzyki, jakim obdarzają nas śpiewające misy.</t>
         </is>
       </c>
       <c r="F346" s="4" t="inlineStr"/>
       <c r="G346" s="5" t="inlineStr"/>
       <c r="H346" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e051"]</t>
+          <t>p[data-content-id="e056"]</t>
         </is>
       </c>
       <c r="I346" s="2" t="inlineStr">
@@ -14117,7 +14117,7 @@
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e052:text</t>
+          <t>terapia-dzwiekiem:e057:text</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
@@ -14137,14 +14137,14 @@
       </c>
       <c r="E347" s="2" t="inlineStr">
         <is>
-          <t>Sesja odbywa się w pozycji leżącej, w ubraniu, które nie krępuje ruchów. Misy mogą być układane w różnych obszarach ciała, między innymi w okolicy stóp, pleców, lędźwi, klatki piersiowej, ramion czy dłoni. Poszczególne elementy masażu dobieram z uwzględnieniem Twoich potrzeb i możliwości. Metoda Petera Hessa® opiera się nie tylko na określonej technice pracy z misami, lecz także na uważności i indywidualnym podejściu do osoby, która z niej korzysta.</t>
+          <t>Zapraszam Cię na indywidualną sesję masażu dźwiękiem metodą Petera Hessa®. To czas, w którym nie musisz niczego robić, nikomu niczego udowadniać ani nigdzie się spieszyć. Możesz po prostu zatrzymać się, odetchnąć i pozwolić, aby dźwięk poprowadził Cię w stronę głębokiego odprężenia, a często także zrozumienia, jakiej zmiany potrzebujesz w swoim życiu.</t>
         </is>
       </c>
       <c r="F347" s="4" t="inlineStr"/>
       <c r="G347" s="5" t="inlineStr"/>
       <c r="H347" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e052"]</t>
+          <t>p[data-content-id="e057"]</t>
         </is>
       </c>
       <c r="I347" s="2" t="inlineStr">
@@ -14156,7 +14156,7 @@
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e053:text</t>
+          <t>terapia-dzwiekiem:e060:href</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
@@ -14171,31 +14171,31 @@
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
         <is>
-          <t>Dźwięki kolejnych mis tworzą harmonię, dzięki której łatwiej zwolnić tempo i skierować uwagę do wewnątrz. Dla wielu osób jest to doświadczenie głębokiego relaksu, pozwalające choć na chwilę odłączyć się od codziennego natłoku myśli i bodźców.</t>
+          <t>index.html#kontakt</t>
         </is>
       </c>
       <c r="F348" s="4" t="inlineStr"/>
       <c r="G348" s="5" t="inlineStr"/>
       <c r="H348" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e053"]</t>
+          <t>a[data-content-id="e060"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I348" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e054:text</t>
+          <t>terapia-dzwiekiem:e060:text</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
@@ -14210,19 +14210,19 @@
       </c>
       <c r="D349" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E349" s="2" t="inlineStr">
         <is>
-          <t>Dlaczego wybrałam Metodę Petera Hessa®?</t>
+          <t>Umów konsultację</t>
         </is>
       </c>
       <c r="F349" s="4" t="inlineStr"/>
       <c r="G349" s="5" t="inlineStr"/>
       <c r="H349" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e054"]</t>
+          <t>a[data-content-id="e060"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I349" s="2" t="inlineStr">
@@ -14234,73 +14234,73 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e055:text</t>
+          <t>warsztaty-i-szkolenia:e006:content</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem.html</t>
+          <t>warsztaty-i-szkolenia.html</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D350" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Opis strony (meta description)</t>
         </is>
       </c>
       <c r="E350" s="2" t="inlineStr">
         <is>
-          <t>Została ona opracowana przez niemieckiego fizyka Petera Hessa na początku lat 80. XX wieku i jest do dziś szeroko wykorzystywana m.in. w obszarze relaksacji, odnowy biologicznej, pedagogiki i pracy wspierającej. Jej ważnym elementem jest indywidualne podejście – sposób prowadzenia masażu może być dostosowany do konkretnej osoby, jej aktualnych potrzeb i możliwości, z uwzględnieniem znajomości fizjologii i biologii ludzkiego ciała.</t>
+          <t>Warsztaty i szkolenia. Praktyczne wsparcie w budowaniu pozycji zawodowej, pewności siebie, skutecznej komunikacji, przywództwa i odporności psychicznej.</t>
         </is>
       </c>
       <c r="F350" s="4" t="inlineStr"/>
       <c r="G350" s="5" t="inlineStr"/>
       <c r="H350" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e055"]</t>
+          <t>meta[data-content-id="e006"]</t>
         </is>
       </c>
       <c r="I350" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>content</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e056:text</t>
+          <t>warsztaty-i-szkolenia:e007:text</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem.html</t>
+          <t>warsztaty-i-szkolenia.html</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D351" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Tytuł strony</t>
         </is>
       </c>
       <c r="E351" s="2" t="inlineStr">
         <is>
-          <t>Metoda ta jest sprawdzona i godna zaufania jako technika relaksacyjna. Nie jest zbiorem sztywnych procedur, ale pozwala na dopasowanie przebiegu spotkania do potrzeb danej osoby i na czerpanie radości z obserwacji, jak wzrasta spokój i harmonia. A wreszcie – jest nieustannym kontaktem z pięknem muzyki, jakim obdarzają nas śpiewające misy.</t>
+          <t>Warsztaty i szkolenia — Katarzyna Chałas</t>
         </is>
       </c>
       <c r="F351" s="4" t="inlineStr"/>
       <c r="G351" s="5" t="inlineStr"/>
       <c r="H351" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e056"]</t>
+          <t>title[data-content-id="e007"]</t>
         </is>
       </c>
       <c r="I351" s="2" t="inlineStr">
@@ -14312,124 +14312,124 @@
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e057:text</t>
+          <t>warsztaty-i-szkolenia:e015:href</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem.html</t>
+          <t>warsztaty-i-szkolenia.html</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E352" s="2" t="inlineStr">
         <is>
-          <t>Zapraszam Cię na indywidualną sesję masażu dźwiękiem metodą Petera Hessa®. To czas, w którym nie musisz niczego robić, nikomu niczego udowadniać ani nigdzie się spieszyć. Możesz po prostu zatrzymać się, odetchnąć i pozwolić, aby dźwięk poprowadził Cię w stronę głębokiego odprężenia, a często także zrozumienia, jakiej zmiany potrzebujesz w swoim życiu.</t>
+          <t>#main-content</t>
         </is>
       </c>
       <c r="F352" s="4" t="inlineStr"/>
       <c r="G352" s="5" t="inlineStr"/>
       <c r="H352" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e057"]</t>
+          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
         </is>
       </c>
       <c r="I352" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e060:href</t>
+          <t>warsztaty-i-szkolenia:e015:text</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem.html</t>
+          <t>warsztaty-i-szkolenia.html</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem</t>
+          <t>Ustawienia strony</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
         <is>
-          <t>index.html#kontakt</t>
+          <t>Przejdź do treści</t>
         </is>
       </c>
       <c r="F353" s="4" t="inlineStr"/>
       <c r="G353" s="5" t="inlineStr"/>
       <c r="H353" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e060"] | Umów konsultację → index.html#kontakt</t>
+          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
         </is>
       </c>
       <c r="I353" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem:e060:text</t>
+          <t>warsztaty-i-szkolenia:e042:href</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>terapia-dzwiekiem.html</t>
+          <t>warsztaty-i-szkolenia.html</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>Terapia dźwiękiem</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E354" s="2" t="inlineStr">
         <is>
-          <t>Umów konsultację</t>
+          <t>index.html</t>
         </is>
       </c>
       <c r="F354" s="4" t="inlineStr"/>
       <c r="G354" s="5" t="inlineStr"/>
       <c r="H354" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e060"] | Umów konsultację → index.html#kontakt</t>
+          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
         </is>
       </c>
       <c r="I354" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e006:content</t>
+          <t>warsztaty-i-szkolenia:e042:text</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
@@ -14439,36 +14439,36 @@
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>Opis strony (meta description)</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
         <is>
-          <t>Warsztaty i szkolenia. Praktyczne wsparcie w budowaniu pozycji zawodowej, pewności siebie, skutecznej komunikacji, przywództwa i odporności psychicznej.</t>
+          <t>← Strona główna</t>
         </is>
       </c>
       <c r="F355" s="4" t="inlineStr"/>
       <c r="G355" s="5" t="inlineStr"/>
       <c r="H355" s="2" t="inlineStr">
         <is>
-          <t>meta[data-content-id="e006"]</t>
+          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
         </is>
       </c>
       <c r="I355" s="2" t="inlineStr">
         <is>
-          <t>content</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e007:text</t>
+          <t>warsztaty-i-szkolenia:e043:text</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
@@ -14478,24 +14478,24 @@
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>Tytuł strony</t>
+          <t>Nagłówek H1</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr">
         <is>
-          <t>Warsztaty i szkolenia — Katarzyna Chałas</t>
+          <t>Warsztaty i szkolenia</t>
         </is>
       </c>
       <c r="F356" s="4" t="inlineStr"/>
       <c r="G356" s="5" t="inlineStr"/>
       <c r="H356" s="2" t="inlineStr">
         <is>
-          <t>title[data-content-id="e007"]</t>
+          <t>h1[data-content-id="e043"]</t>
         </is>
       </c>
       <c r="I356" s="2" t="inlineStr">
@@ -14507,7 +14507,7 @@
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e015:href</t>
+          <t>warsztaty-i-szkolenia:e044:text</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
@@ -14517,36 +14517,36 @@
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr">
         <is>
-          <t>#main-content</t>
+          <t>Praktyczne wsparcie w budowaniu pozycji zawodowej, pewności siebie, skutecznej komunikacji i odporności psychicznej, a także prowadzenie przez zmianę i wdrażanie zmian.</t>
         </is>
       </c>
       <c r="F357" s="4" t="inlineStr"/>
       <c r="G357" s="5" t="inlineStr"/>
       <c r="H357" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
+          <t>p[data-content-id="e044"]</t>
         </is>
       </c>
       <c r="I357" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e015:text</t>
+          <t>warsztaty-i-szkolenia:e046:alt</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
@@ -14556,36 +14556,36 @@
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>Ustawienia strony</t>
+          <t>Banner</t>
         </is>
       </c>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Opis obrazu (alt)</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr">
         <is>
-          <t>Przejdź do treści</t>
+          <t>Katarzyna Chałas - coach</t>
         </is>
       </c>
       <c r="F358" s="4" t="inlineStr"/>
       <c r="G358" s="5" t="inlineStr"/>
       <c r="H358" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e015"] | Przejdź do treści → #main-content</t>
+          <t>img[data-content-id="e046"] | assets/hero-warsztaty-1000.webp</t>
         </is>
       </c>
       <c r="I358" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>alt</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e042:href</t>
+          <t>warsztaty-i-szkolenia:e049:text</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
@@ -14595,36 +14595,36 @@
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Warsztaty i szkolenia</t>
         </is>
       </c>
       <c r="D359" s="2" t="inlineStr">
         <is>
-          <t>Adres linku</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E359" s="2" t="inlineStr">
         <is>
-          <t>index.html</t>
+          <t>Dla rozwoju czasami kluczowe jest lepsze zrozumienie, co wpływa na nasze sposoby działania, jak funkcjonuje człowiek i czego potrzeba, by skutecznie radzić sobie z wyzwaniami – zawodowymi i osobistymi. Dlatego prowadzę szkolenia i warsztaty, które łączą wiedzę z psychologii biznesu z praktyczną pracą nad zachowaniami, przekonaniami i sposobami funkcjonowania w środowisku zawodowym i życiu osobistym.</t>
         </is>
       </c>
       <c r="F359" s="4" t="inlineStr"/>
       <c r="G359" s="5" t="inlineStr"/>
       <c r="H359" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>p[data-content-id="e049"]</t>
         </is>
       </c>
       <c r="I359" s="2" t="inlineStr">
         <is>
-          <t>href</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e042:text</t>
+          <t>warsztaty-i-szkolenia:e083:text</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
@@ -14634,24 +14634,24 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Warsztaty i szkolenia</t>
         </is>
       </c>
       <c r="D360" s="2" t="inlineStr">
         <is>
-          <t>Etykieta linku</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E360" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Focus na odporność psychiczną i wellbeing kobiet</t>
         </is>
       </c>
       <c r="F360" s="4" t="inlineStr"/>
       <c r="G360" s="5" t="inlineStr"/>
       <c r="H360" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>h2[data-content-id="e083"]</t>
         </is>
       </c>
       <c r="I360" s="2" t="inlineStr">
@@ -14663,7 +14663,7 @@
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e043:text</t>
+          <t>warsztaty-i-szkolenia:e084:text</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
@@ -14673,24 +14673,24 @@
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Warsztaty i szkolenia</t>
         </is>
       </c>
       <c r="D361" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H1</t>
+          <t>Akapit</t>
         </is>
       </c>
       <c r="E361" s="2" t="inlineStr">
         <is>
-          <t>Warsztaty i szkolenia</t>
+          <t>Jednym z ważnych dla mnie obszarów jest odporność psychiczna, rozumiana nie jako obowiązek „bycia silnym bez względu na wszystko”, ale jako umiejętność świadomego radzenia sobie z wyzwaniami, stresem i niepewnością. Szczególną uwagę kieruję do kobiet i mężczyzn 55+ i ich utrzymywania aktywności na rynku pracy.</t>
         </is>
       </c>
       <c r="F361" s="4" t="inlineStr"/>
       <c r="G361" s="5" t="inlineStr"/>
       <c r="H361" s="2" t="inlineStr">
         <is>
-          <t>h1[data-content-id="e043"]</t>
+          <t>p[data-content-id="e084"]</t>
         </is>
       </c>
       <c r="I361" s="2" t="inlineStr">
@@ -14702,7 +14702,7 @@
     <row r="362">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e044:text</t>
+          <t>warsztaty-i-szkolenia:e085:text</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
@@ -14712,7 +14712,7 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Warsztaty i szkolenia</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr">
@@ -14722,14 +14722,14 @@
       </c>
       <c r="E362" s="2" t="inlineStr">
         <is>
-          <t>Praktyczne wsparcie w budowaniu pozycji zawodowej, pewności siebie, skutecznej komunikacji i odporności psychicznej, a także prowadzenie przez zmianę i wdrażanie zmian.</t>
+          <t>Moje programy rozwojowe z zakresu odporności psychicznej, budowania pewności siebie i pozycji zawodowej w specjalny sposób kieruję do kobiet – jestem organizatorką serii warsztatów m.in. o pieniądzach, zdrowiu, kreatywności. Inspirujące spotkania w kobiecym gronie niejednokrotnie odbywają się przy kojących dźwiękach mis tybetańskich.</t>
         </is>
       </c>
       <c r="F362" s="4" t="inlineStr"/>
       <c r="G362" s="5" t="inlineStr"/>
       <c r="H362" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e044"]</t>
+          <t>p[data-content-id="e085"]</t>
         </is>
       </c>
       <c r="I362" s="2" t="inlineStr">
@@ -14741,7 +14741,7 @@
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e046:alt</t>
+          <t>warsztaty-i-szkolenia:e086:text</t>
         </is>
       </c>
       <c r="B363" s="2" t="inlineStr">
@@ -14751,36 +14751,36 @@
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>Banner</t>
+          <t>Warsztaty i szkolenia</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr">
         <is>
-          <t>Opis obrazu (alt)</t>
+          <t>Nagłówek H2</t>
         </is>
       </c>
       <c r="E363" s="2" t="inlineStr">
         <is>
-          <t>Katarzyna Chałas - coach</t>
+          <t>Jak pracuję?</t>
         </is>
       </c>
       <c r="F363" s="4" t="inlineStr"/>
       <c r="G363" s="5" t="inlineStr"/>
       <c r="H363" s="2" t="inlineStr">
         <is>
-          <t>img[data-content-id="e046"] | assets/hero-warsztaty-1000.webp</t>
+          <t>h2[data-content-id="e086"]</t>
         </is>
       </c>
       <c r="I363" s="2" t="inlineStr">
         <is>
-          <t>alt</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e049:text</t>
+          <t>warsztaty-i-szkolenia:e087:text</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
@@ -14800,14 +14800,14 @@
       </c>
       <c r="E364" s="2" t="inlineStr">
         <is>
-          <t>Dla rozwoju czasami kluczowe jest lepsze zrozumienie, co wpływa na nasze sposoby działania, jak funkcjonuje człowiek i czego potrzeba, by skutecznie radzić sobie z wyzwaniami – zawodowymi i osobistymi. Dlatego prowadzę szkolenia i warsztaty, które łączą wiedzę z psychologii biznesu z praktyczną pracą nad zachowaniami, przekonaniami i sposobami funkcjonowania w środowisku zawodowym i życiu osobistym.</t>
+          <t>Nie zależy mi na spotkaniu, po którym uczestnicy wychodzą jedynie z notesem pełnym haseł. Wiedza jest dla mnie punktem wyjścia. Celem – to, co można z nią zrobić. Dlatego w szkoleniach łączę krótkie wprowadzenie merytoryczne z pracą warsztatową, uczeniem zadawania odpowiednich pytań, analizą rzeczywistych sytuacji oraz wymianą doświadczeń. Tam, gdzie jest to uzasadnione, wspieram uczestników narzędziami diagnostycznymi i psychometrycznymi.</t>
         </is>
       </c>
       <c r="F364" s="4" t="inlineStr"/>
       <c r="G364" s="5" t="inlineStr"/>
       <c r="H364" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e049"]</t>
+          <t>p[data-content-id="e087"]</t>
         </is>
       </c>
       <c r="I364" s="2" t="inlineStr">
@@ -14819,7 +14819,7 @@
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e083:text</t>
+          <t>warsztaty-i-szkolenia:e088:text</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
@@ -14839,14 +14839,14 @@
       </c>
       <c r="E365" s="2" t="inlineStr">
         <is>
-          <t>Focus na odporność psychiczną i wellbeing kobiet</t>
+          <t>Szkolenie dopasowane do rzeczywistej potrzeby</t>
         </is>
       </c>
       <c r="F365" s="4" t="inlineStr"/>
       <c r="G365" s="5" t="inlineStr"/>
       <c r="H365" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e083"]</t>
+          <t>h2[data-content-id="e088"]</t>
         </is>
       </c>
       <c r="I365" s="2" t="inlineStr">
@@ -14858,7 +14858,7 @@
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e084:text</t>
+          <t>warsztaty-i-szkolenia:e089:text</t>
         </is>
       </c>
       <c r="B366" s="2" t="inlineStr">
@@ -14878,14 +14878,14 @@
       </c>
       <c r="E366" s="2" t="inlineStr">
         <is>
-          <t>Jednym z ważnych dla mnie obszarów jest odporność psychiczna, rozumiana nie jako obowiązek „bycia silnym bez względu na wszystko”, ale jako umiejętność świadomego radzenia sobie z wyzwaniami, stresem i niepewnością. Szczególną uwagę kieruję do kobiet i mężczyzn 55+ i ich utrzymywania aktywności na rynku pracy.</t>
+          <t>Prowadzone przeze mnie warsztaty są każdorazowo dopasowywane do potrzeb pod kątem tematyki, zakresu i formy.</t>
         </is>
       </c>
       <c r="F366" s="4" t="inlineStr"/>
       <c r="G366" s="5" t="inlineStr"/>
       <c r="H366" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e084"]</t>
+          <t>p[data-content-id="e089"]</t>
         </is>
       </c>
       <c r="I366" s="2" t="inlineStr">
@@ -14897,7 +14897,7 @@
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e085:text</t>
+          <t>warsztaty-i-szkolenia:e090:text</t>
         </is>
       </c>
       <c r="B367" s="2" t="inlineStr">
@@ -14917,14 +14917,14 @@
       </c>
       <c r="E367" s="2" t="inlineStr">
         <is>
-          <t>Moje programy rozwojowe z zakresu odporności psychicznej, budowania pewności siebie i pozycji zawodowej w specjalny sposób kieruję do kobiet – jestem organizatorką serii warsztatów m.in. o pieniądzach, zdrowiu, kreatywności. Inspirujące spotkania w kobiecym gronie niejednokrotnie odbywają się przy kojących dźwiękach mis tybetańskich.</t>
+          <t>Jeśli szukasz warsztatów, w których inspiracja zostaje przekuta w świadomość i rzeczywistą zmianę, porozmawiajmy!</t>
         </is>
       </c>
       <c r="F367" s="4" t="inlineStr"/>
       <c r="G367" s="5" t="inlineStr"/>
       <c r="H367" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e085"]</t>
+          <t>p[data-content-id="e090"]</t>
         </is>
       </c>
       <c r="I367" s="2" t="inlineStr">
@@ -14936,7 +14936,7 @@
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e086:text</t>
+          <t>warsztaty-i-szkolenia:e093:href</t>
         </is>
       </c>
       <c r="B368" s="2" t="inlineStr">
@@ -14951,31 +14951,31 @@
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>Nagłówek H2</t>
+          <t>Adres linku</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
         <is>
-          <t>Jak pracuję?</t>
+          <t>index.html#kontakt</t>
         </is>
       </c>
       <c r="F368" s="4" t="inlineStr"/>
       <c r="G368" s="5" t="inlineStr"/>
       <c r="H368" s="2" t="inlineStr">
         <is>
-          <t>h2[data-content-id="e086"]</t>
+          <t>a[data-content-id="e093"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I368" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>href</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>warsztaty-i-szkolenia:e087:text</t>
+          <t>warsztaty-i-szkolenia:e093:text</t>
         </is>
       </c>
       <c r="B369" s="2" t="inlineStr">
@@ -14990,19 +14990,19 @@
       </c>
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>Akapit</t>
+          <t>Etykieta linku</t>
         </is>
       </c>
       <c r="E369" s="2" t="inlineStr">
         <is>
-          <t>Nie zależy mi na spotkaniu, po którym uczestnicy wychodzą jedynie z notesem pełnym haseł. Wiedza jest dla mnie punktem wyjścia. Celem – to, co można z nią zrobić. Dlatego w szkoleniach łączę krótkie wprowadzenie merytoryczne z pracą warsztatową, uczeniem zadawania odpowiednich pytań, analizą rzeczywistych sytuacji oraz wymianą doświadczeń. Tam, gdzie jest to uzasadnione, wspieram uczestników narzędziami diagnostycznymi i psychometrycznymi.</t>
+          <t>Umów konsultację</t>
         </is>
       </c>
       <c r="F369" s="4" t="inlineStr"/>
       <c r="G369" s="5" t="inlineStr"/>
       <c r="H369" s="2" t="inlineStr">
         <is>
-          <t>p[data-content-id="e087"]</t>
+          <t>a[data-content-id="e093"] | Umów konsultację → index.html#kontakt</t>
         </is>
       </c>
       <c r="I369" s="2" t="inlineStr">
@@ -15011,203 +15011,8 @@
         </is>
       </c>
     </row>
-    <row r="370">
-      <c r="A370" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia:e088:text</t>
-        </is>
-      </c>
-      <c r="B370" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia.html</t>
-        </is>
-      </c>
-      <c r="C370" s="2" t="inlineStr">
-        <is>
-          <t>Warsztaty i szkolenia</t>
-        </is>
-      </c>
-      <c r="D370" s="2" t="inlineStr">
-        <is>
-          <t>Nagłówek H2</t>
-        </is>
-      </c>
-      <c r="E370" s="2" t="inlineStr">
-        <is>
-          <t>Szkolenie dopasowane do rzeczywistej potrzeby</t>
-        </is>
-      </c>
-      <c r="F370" s="4" t="inlineStr"/>
-      <c r="G370" s="5" t="inlineStr"/>
-      <c r="H370" s="2" t="inlineStr">
-        <is>
-          <t>h2[data-content-id="e088"]</t>
-        </is>
-      </c>
-      <c r="I370" s="2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia:e089:text</t>
-        </is>
-      </c>
-      <c r="B371" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia.html</t>
-        </is>
-      </c>
-      <c r="C371" s="2" t="inlineStr">
-        <is>
-          <t>Warsztaty i szkolenia</t>
-        </is>
-      </c>
-      <c r="D371" s="2" t="inlineStr">
-        <is>
-          <t>Akapit</t>
-        </is>
-      </c>
-      <c r="E371" s="2" t="inlineStr">
-        <is>
-          <t>Prowadzone przeze mnie warsztaty są każdorazowo dopasowywane do potrzeb pod kątem tematyki, zakresu i formy.</t>
-        </is>
-      </c>
-      <c r="F371" s="4" t="inlineStr"/>
-      <c r="G371" s="5" t="inlineStr"/>
-      <c r="H371" s="2" t="inlineStr">
-        <is>
-          <t>p[data-content-id="e089"]</t>
-        </is>
-      </c>
-      <c r="I371" s="2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia:e090:text</t>
-        </is>
-      </c>
-      <c r="B372" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia.html</t>
-        </is>
-      </c>
-      <c r="C372" s="2" t="inlineStr">
-        <is>
-          <t>Warsztaty i szkolenia</t>
-        </is>
-      </c>
-      <c r="D372" s="2" t="inlineStr">
-        <is>
-          <t>Akapit</t>
-        </is>
-      </c>
-      <c r="E372" s="2" t="inlineStr">
-        <is>
-          <t>Jeśli szukasz warsztatów, w których inspiracja zostaje przekuta w świadomość i rzeczywistą zmianę, porozmawiajmy!</t>
-        </is>
-      </c>
-      <c r="F372" s="4" t="inlineStr"/>
-      <c r="G372" s="5" t="inlineStr"/>
-      <c r="H372" s="2" t="inlineStr">
-        <is>
-          <t>p[data-content-id="e090"]</t>
-        </is>
-      </c>
-      <c r="I372" s="2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia:e093:href</t>
-        </is>
-      </c>
-      <c r="B373" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia.html</t>
-        </is>
-      </c>
-      <c r="C373" s="2" t="inlineStr">
-        <is>
-          <t>Warsztaty i szkolenia</t>
-        </is>
-      </c>
-      <c r="D373" s="2" t="inlineStr">
-        <is>
-          <t>Adres linku</t>
-        </is>
-      </c>
-      <c r="E373" s="2" t="inlineStr">
-        <is>
-          <t>index.html#kontakt</t>
-        </is>
-      </c>
-      <c r="F373" s="4" t="inlineStr"/>
-      <c r="G373" s="5" t="inlineStr"/>
-      <c r="H373" s="2" t="inlineStr">
-        <is>
-          <t>a[data-content-id="e093"] | Umów konsultację → index.html#kontakt</t>
-        </is>
-      </c>
-      <c r="I373" s="2" t="inlineStr">
-        <is>
-          <t>href</t>
-        </is>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia:e093:text</t>
-        </is>
-      </c>
-      <c r="B374" s="2" t="inlineStr">
-        <is>
-          <t>warsztaty-i-szkolenia.html</t>
-        </is>
-      </c>
-      <c r="C374" s="2" t="inlineStr">
-        <is>
-          <t>Warsztaty i szkolenia</t>
-        </is>
-      </c>
-      <c r="D374" s="2" t="inlineStr">
-        <is>
-          <t>Etykieta linku</t>
-        </is>
-      </c>
-      <c r="E374" s="2" t="inlineStr">
-        <is>
-          <t>Umów konsultację</t>
-        </is>
-      </c>
-      <c r="F374" s="4" t="inlineStr"/>
-      <c r="G374" s="5" t="inlineStr"/>
-      <c r="H374" s="2" t="inlineStr">
-        <is>
-          <t>a[data-content-id="e093"] | Umów konsultację → index.html#kontakt</t>
-        </is>
-      </c>
-      <c r="I374" s="2" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I374"/>
+  <autoFilter ref="A1:I369"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Complete font sizing and SVG back links for cards 1933 and 1934
</commit_message>
<xml_diff>
--- a/teksty-strony.xlsx
+++ b/teksty-strony.xlsx
@@ -6383,7 +6383,7 @@
       <c r="G148" s="5" t="inlineStr"/>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I148" s="2" t="inlineStr">
@@ -6415,14 +6415,14 @@
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F149" s="4" t="inlineStr"/>
       <c r="G149" s="5" t="inlineStr"/>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I149" s="2" t="inlineStr">
@@ -7514,7 +7514,7 @@
       <c r="G177" s="5" t="inlineStr"/>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I177" s="2" t="inlineStr">
@@ -7546,14 +7546,14 @@
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F178" s="4" t="inlineStr"/>
       <c r="G178" s="5" t="inlineStr"/>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I178" s="2" t="inlineStr">
@@ -8333,7 +8333,7 @@
       <c r="G198" s="5" t="inlineStr"/>
       <c r="H198" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I198" s="2" t="inlineStr">
@@ -8365,14 +8365,14 @@
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F199" s="4" t="inlineStr"/>
       <c r="G199" s="5" t="inlineStr"/>
       <c r="H199" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I199" s="2" t="inlineStr">
@@ -9347,7 +9347,7 @@
       <c r="G224" s="5" t="inlineStr"/>
       <c r="H224" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I224" s="2" t="inlineStr">
@@ -9379,14 +9379,14 @@
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F225" s="4" t="inlineStr"/>
       <c r="G225" s="5" t="inlineStr"/>
       <c r="H225" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I225" s="2" t="inlineStr">
@@ -11531,7 +11531,7 @@
       <c r="G280" s="5" t="inlineStr"/>
       <c r="H280" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I280" s="2" t="inlineStr">
@@ -11563,14 +11563,14 @@
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F281" s="4" t="inlineStr"/>
       <c r="G281" s="5" t="inlineStr"/>
       <c r="H281" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I281" s="2" t="inlineStr">
@@ -12584,7 +12584,7 @@
       <c r="G307" s="5" t="inlineStr"/>
       <c r="H307" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I307" s="2" t="inlineStr">
@@ -12616,14 +12616,14 @@
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F308" s="4" t="inlineStr"/>
       <c r="G308" s="5" t="inlineStr"/>
       <c r="H308" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I308" s="2" t="inlineStr">
@@ -13637,7 +13637,7 @@
       <c r="G334" s="5" t="inlineStr"/>
       <c r="H334" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I334" s="2" t="inlineStr">
@@ -13669,14 +13669,14 @@
       </c>
       <c r="E335" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F335" s="4" t="inlineStr"/>
       <c r="G335" s="5" t="inlineStr"/>
       <c r="H335" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I335" s="2" t="inlineStr">
@@ -14417,7 +14417,7 @@
       <c r="G354" s="5" t="inlineStr"/>
       <c r="H354" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I354" s="2" t="inlineStr">
@@ -14449,14 +14449,14 @@
       </c>
       <c r="E355" s="2" t="inlineStr">
         <is>
-          <t>← Strona główna</t>
+          <t>Strona główna</t>
         </is>
       </c>
       <c r="F355" s="4" t="inlineStr"/>
       <c r="G355" s="5" t="inlineStr"/>
       <c r="H355" s="2" t="inlineStr">
         <is>
-          <t>a[data-content-id="e042"] | ← Strona główna → index.html</t>
+          <t>a[data-content-id="e042"] | Strona główna → index.html</t>
         </is>
       </c>
       <c r="I355" s="2" t="inlineStr">

</xml_diff>